<commit_message>
Lo 02 dinh danh: anh Lam duyet 'da duyet va xac nhan thong qua' (duyet.json), nap 55 claim (43 ten_phap_nhan, 12 ma_so_tu_khai) vao registry, 9 muc can anh quyet giu trong. Hai truong dinh danh tu khai trong domain.yaml, BEN trong do tuoi, khong vao dong thoi gian/thoi cuoc/bieu do theo nam. Web: ho so va so nguon hien 'Tu khai, chua doi chieu cong', khong doi trang thai dinh danh (cong TU_KHAI_LECH, TU_KHAI_THANH_DINH_DANH + 2 rang). check_ngay_dang: luat TRANG TINH cho truong dinh danh + 3 rang. Duong tra cong: nap_tra_cong.py (PDF phai mang dau cong, dung ma, dung ten) + 12 rang; check_ma_so_thue giu nguyen. bite_kiem_lo dung canh dung khi co lo nap sau. Trang dau, tong quan ghi ro luot kiem nhanh. Chuoi nhanh 61/61 + 42 rang xanh (chay tach hai phan), axe 0.
</commit_message>
<xml_diff>
--- a/CNCLData/lam_giau/dot_02/PHIEU_TRA_CONG.xlsx
+++ b/CNCLData/lam_giau/dot_02/PHIEU_TRA_CONG.xlsx
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="311">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="312">
   <si>
     <t xml:space="preserve">Phiếu tra cổng · định danh pháp nhân</t>
   </si>
@@ -76,6 +76,9 @@
   </si>
   <si>
     <t xml:space="preserve">Chỉ sửa ô VÀNG. Dòng 3 của tab "Phiếu tra" là dòng MẪU (in nghiêng), không phải dữ liệu thật.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tra xong: lưu file này, báo người vận hành chạy nap_tra_cong.py. Máy chỉ nạp dòng có PDF mang dấu cổng, đúng mã và đúng tên đã ghi.</t>
   </si>
   <si>
     <t xml:space="preserve">STT</t>
@@ -1404,7 +1407,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A14"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
@@ -1472,6 +1475,11 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="2" t="s">
         <v>10</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -1510,99 +1518,99 @@
   <sheetData>
     <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E3" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" s="5" t="s">
-        <v>30</v>
-      </c>
       <c r="I3" s="5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="K3" s="5" t="str">
         <f aca="false">IF(H3="","",IF(D3="","CHỈ CÓ MÃ CỔNG",IF(TRIM(H3)=TRIM(D3),"KHỚP","LỆCH")))</f>
         <v>KHỚP</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="O3" s="5"/>
     </row>
@@ -1611,20 +1619,20 @@
         <v>1</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D4" s="7"/>
       <c r="E4" s="6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H4" s="8"/>
       <c r="I4" s="9"/>
@@ -1636,7 +1644,7 @@
       <c r="L4" s="9"/>
       <c r="M4" s="9"/>
       <c r="N4" s="10" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="O4" s="9"/>
     </row>
@@ -1645,22 +1653,22 @@
         <v>2</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="H5" s="8"/>
       <c r="I5" s="9"/>
@@ -1672,7 +1680,7 @@
       <c r="L5" s="9"/>
       <c r="M5" s="9"/>
       <c r="N5" s="10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="O5" s="9"/>
     </row>
@@ -1681,20 +1689,20 @@
         <v>3</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H6" s="8"/>
       <c r="I6" s="9"/>
@@ -1706,7 +1714,7 @@
       <c r="L6" s="9"/>
       <c r="M6" s="9"/>
       <c r="N6" s="10" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="O6" s="9"/>
     </row>
@@ -1715,14 +1723,14 @@
         <v>4</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7"/>
       <c r="E7" s="6"/>
       <c r="F7" s="6"/>
       <c r="G7" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="9"/>
@@ -1734,7 +1742,7 @@
       <c r="L7" s="9"/>
       <c r="M7" s="9"/>
       <c r="N7" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="O7" s="9"/>
     </row>
@@ -1743,18 +1751,18 @@
         <v>5</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D8" s="7"/>
       <c r="E8" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H8" s="8"/>
       <c r="I8" s="9"/>
@@ -1766,7 +1774,7 @@
       <c r="L8" s="9"/>
       <c r="M8" s="9"/>
       <c r="N8" s="10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="O8" s="9"/>
     </row>
@@ -1775,22 +1783,22 @@
         <v>6</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D9" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H9" s="8"/>
       <c r="I9" s="9"/>
@@ -1802,7 +1810,7 @@
       <c r="L9" s="9"/>
       <c r="M9" s="9"/>
       <c r="N9" s="10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="O9" s="9"/>
     </row>
@@ -1811,18 +1819,18 @@
         <v>7</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D10" s="7"/>
       <c r="E10" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H10" s="8"/>
       <c r="I10" s="9"/>
@@ -1834,7 +1842,7 @@
       <c r="L10" s="9"/>
       <c r="M10" s="9"/>
       <c r="N10" s="10" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="O10" s="9"/>
     </row>
@@ -1843,18 +1851,18 @@
         <v>8</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D11" s="7"/>
       <c r="E11" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H11" s="8"/>
       <c r="I11" s="9"/>
@@ -1866,7 +1874,7 @@
       <c r="L11" s="9"/>
       <c r="M11" s="9"/>
       <c r="N11" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="O11" s="9"/>
     </row>
@@ -1875,14 +1883,14 @@
         <v>9</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C12" s="6"/>
       <c r="D12" s="7"/>
       <c r="E12" s="6"/>
       <c r="F12" s="6"/>
       <c r="G12" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H12" s="8"/>
       <c r="I12" s="9"/>
@@ -1894,7 +1902,7 @@
       <c r="L12" s="9"/>
       <c r="M12" s="9"/>
       <c r="N12" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="O12" s="9"/>
     </row>
@@ -1903,18 +1911,18 @@
         <v>10</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D13" s="7"/>
       <c r="E13" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H13" s="8"/>
       <c r="I13" s="9"/>
@@ -1926,7 +1934,7 @@
       <c r="L13" s="9"/>
       <c r="M13" s="9"/>
       <c r="N13" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O13" s="9"/>
     </row>
@@ -1935,18 +1943,18 @@
         <v>11</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D14" s="7"/>
       <c r="E14" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H14" s="8"/>
       <c r="I14" s="9"/>
@@ -1958,7 +1966,7 @@
       <c r="L14" s="9"/>
       <c r="M14" s="9"/>
       <c r="N14" s="10" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O14" s="9"/>
     </row>
@@ -1967,22 +1975,22 @@
         <v>12</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H15" s="8"/>
       <c r="I15" s="9"/>
@@ -1994,7 +2002,7 @@
       <c r="L15" s="9"/>
       <c r="M15" s="9"/>
       <c r="N15" s="10" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="O15" s="9"/>
     </row>
@@ -2003,18 +2011,18 @@
         <v>13</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D16" s="7"/>
       <c r="E16" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F16" s="6"/>
       <c r="G16" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H16" s="8"/>
       <c r="I16" s="9"/>
@@ -2026,7 +2034,7 @@
       <c r="L16" s="9"/>
       <c r="M16" s="9"/>
       <c r="N16" s="10" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="O16" s="9"/>
     </row>
@@ -2035,20 +2043,20 @@
         <v>14</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D17" s="7"/>
       <c r="E17" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H17" s="8"/>
       <c r="I17" s="9"/>
@@ -2060,7 +2068,7 @@
       <c r="L17" s="9"/>
       <c r="M17" s="9"/>
       <c r="N17" s="10" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="O17" s="9"/>
     </row>
@@ -2069,20 +2077,20 @@
         <v>15</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="D18" s="7"/>
       <c r="E18" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H18" s="8"/>
       <c r="I18" s="9"/>
@@ -2094,7 +2102,7 @@
       <c r="L18" s="9"/>
       <c r="M18" s="9"/>
       <c r="N18" s="10" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="O18" s="9"/>
     </row>
@@ -2103,14 +2111,14 @@
         <v>16</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="7"/>
       <c r="E19" s="6"/>
       <c r="F19" s="6"/>
       <c r="G19" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H19" s="8"/>
       <c r="I19" s="9"/>
@@ -2122,7 +2130,7 @@
       <c r="L19" s="9"/>
       <c r="M19" s="9"/>
       <c r="N19" s="10" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="O19" s="9"/>
     </row>
@@ -2131,16 +2139,16 @@
         <v>17</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="7"/>
       <c r="E20" s="6"/>
       <c r="F20" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="9"/>
@@ -2152,7 +2160,7 @@
       <c r="L20" s="9"/>
       <c r="M20" s="9"/>
       <c r="N20" s="10" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="O20" s="9"/>
     </row>
@@ -2161,18 +2169,18 @@
         <v>18</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D21" s="7"/>
       <c r="E21" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H21" s="8"/>
       <c r="I21" s="9"/>
@@ -2184,7 +2192,7 @@
       <c r="L21" s="9"/>
       <c r="M21" s="9"/>
       <c r="N21" s="10" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="O21" s="9"/>
     </row>
@@ -2193,20 +2201,20 @@
         <v>19</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="9"/>
@@ -2218,7 +2226,7 @@
       <c r="L22" s="9"/>
       <c r="M22" s="9"/>
       <c r="N22" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="O22" s="9"/>
     </row>
@@ -2227,20 +2235,20 @@
         <v>20</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H23" s="8"/>
       <c r="I23" s="9"/>
@@ -2252,7 +2260,7 @@
       <c r="L23" s="9"/>
       <c r="M23" s="9"/>
       <c r="N23" s="10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="O23" s="9"/>
     </row>
@@ -2261,14 +2269,14 @@
         <v>21</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="7"/>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
       <c r="G24" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H24" s="8"/>
       <c r="I24" s="9"/>
@@ -2280,7 +2288,7 @@
       <c r="L24" s="9"/>
       <c r="M24" s="9"/>
       <c r="N24" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="O24" s="9"/>
     </row>
@@ -2289,18 +2297,18 @@
         <v>22</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D25" s="7"/>
       <c r="E25" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H25" s="8"/>
       <c r="I25" s="9"/>
@@ -2312,7 +2320,7 @@
       <c r="L25" s="9"/>
       <c r="M25" s="9"/>
       <c r="N25" s="10" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="O25" s="9"/>
     </row>
@@ -2321,18 +2329,18 @@
         <v>23</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D26" s="7"/>
       <c r="E26" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F26" s="6"/>
       <c r="G26" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H26" s="8"/>
       <c r="I26" s="9"/>
@@ -2344,7 +2352,7 @@
       <c r="L26" s="9"/>
       <c r="M26" s="9"/>
       <c r="N26" s="10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="O26" s="9"/>
     </row>
@@ -2353,16 +2361,16 @@
         <v>24</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
       <c r="E27" s="6"/>
       <c r="F27" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="9"/>
@@ -2374,7 +2382,7 @@
       <c r="L27" s="9"/>
       <c r="M27" s="9"/>
       <c r="N27" s="10" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="O27" s="9"/>
     </row>
@@ -2383,14 +2391,14 @@
         <v>25</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
       <c r="E28" s="6"/>
       <c r="F28" s="6"/>
       <c r="G28" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H28" s="8"/>
       <c r="I28" s="9"/>
@@ -2402,7 +2410,7 @@
       <c r="L28" s="9"/>
       <c r="M28" s="9"/>
       <c r="N28" s="10" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="O28" s="9"/>
     </row>
@@ -2411,20 +2419,20 @@
         <v>26</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F29" s="6"/>
       <c r="G29" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H29" s="8"/>
       <c r="I29" s="9"/>
@@ -2436,7 +2444,7 @@
       <c r="L29" s="9"/>
       <c r="M29" s="9"/>
       <c r="N29" s="10" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="O29" s="9"/>
     </row>
@@ -2445,14 +2453,14 @@
         <v>27</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="7"/>
       <c r="E30" s="6"/>
       <c r="F30" s="6"/>
       <c r="G30" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="H30" s="8"/>
       <c r="I30" s="9"/>
@@ -2464,7 +2472,7 @@
       <c r="L30" s="9"/>
       <c r="M30" s="9"/>
       <c r="N30" s="10" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="O30" s="9"/>
     </row>
@@ -2473,18 +2481,18 @@
         <v>28</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D31" s="7"/>
       <c r="E31" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H31" s="8"/>
       <c r="I31" s="9"/>
@@ -2496,7 +2504,7 @@
       <c r="L31" s="9"/>
       <c r="M31" s="9"/>
       <c r="N31" s="10" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="O31" s="9"/>
     </row>
@@ -2505,14 +2513,14 @@
         <v>29</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
       <c r="E32" s="6"/>
       <c r="F32" s="6"/>
       <c r="G32" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H32" s="8"/>
       <c r="I32" s="9"/>
@@ -2524,7 +2532,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="9"/>
       <c r="N32" s="10" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="O32" s="9"/>
     </row>
@@ -2533,14 +2541,14 @@
         <v>30</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
       <c r="E33" s="6"/>
       <c r="F33" s="6"/>
       <c r="G33" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H33" s="8"/>
       <c r="I33" s="9"/>
@@ -2552,7 +2560,7 @@
       <c r="L33" s="9"/>
       <c r="M33" s="9"/>
       <c r="N33" s="10" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="O33" s="9"/>
     </row>
@@ -2561,20 +2569,20 @@
         <v>31</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H34" s="8"/>
       <c r="I34" s="9"/>
@@ -2586,7 +2594,7 @@
       <c r="L34" s="9"/>
       <c r="M34" s="9"/>
       <c r="N34" s="10" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="O34" s="9"/>
     </row>
@@ -2595,20 +2603,20 @@
         <v>32</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D35" s="7"/>
       <c r="E35" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H35" s="8"/>
       <c r="I35" s="9"/>
@@ -2620,7 +2628,7 @@
       <c r="L35" s="9"/>
       <c r="M35" s="9"/>
       <c r="N35" s="10" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="O35" s="9"/>
     </row>
@@ -2629,18 +2637,18 @@
         <v>33</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H36" s="8"/>
       <c r="I36" s="9"/>
@@ -2652,7 +2660,7 @@
       <c r="L36" s="9"/>
       <c r="M36" s="9"/>
       <c r="N36" s="10" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="O36" s="9"/>
     </row>
@@ -2661,22 +2669,22 @@
         <v>34</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H37" s="8"/>
       <c r="I37" s="9"/>
@@ -2688,7 +2696,7 @@
       <c r="L37" s="9"/>
       <c r="M37" s="9"/>
       <c r="N37" s="10" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="O37" s="9"/>
     </row>
@@ -2697,20 +2705,20 @@
         <v>35</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="9"/>
@@ -2722,7 +2730,7 @@
       <c r="L38" s="9"/>
       <c r="M38" s="9"/>
       <c r="N38" s="10" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="O38" s="9"/>
     </row>
@@ -2731,20 +2739,20 @@
         <v>36</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H39" s="8"/>
       <c r="I39" s="9"/>
@@ -2756,7 +2764,7 @@
       <c r="L39" s="9"/>
       <c r="M39" s="9"/>
       <c r="N39" s="10" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O39" s="9"/>
     </row>
@@ -2765,20 +2773,20 @@
         <v>37</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D40" s="7" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H40" s="8"/>
       <c r="I40" s="9"/>
@@ -2790,7 +2798,7 @@
       <c r="L40" s="9"/>
       <c r="M40" s="9"/>
       <c r="N40" s="10" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="O40" s="9"/>
     </row>
@@ -2799,20 +2807,20 @@
         <v>38</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="H41" s="8"/>
       <c r="I41" s="9"/>
@@ -2824,7 +2832,7 @@
       <c r="L41" s="9"/>
       <c r="M41" s="9"/>
       <c r="N41" s="10" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="O41" s="9"/>
     </row>
@@ -2833,20 +2841,20 @@
         <v>39</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H42" s="8"/>
       <c r="I42" s="9"/>
@@ -2858,7 +2866,7 @@
       <c r="L42" s="9"/>
       <c r="M42" s="9"/>
       <c r="N42" s="10" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="O42" s="9"/>
     </row>
@@ -2867,20 +2875,20 @@
         <v>40</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H43" s="8"/>
       <c r="I43" s="9"/>
@@ -2892,7 +2900,7 @@
       <c r="L43" s="9"/>
       <c r="M43" s="9"/>
       <c r="N43" s="10" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="O43" s="9"/>
     </row>
@@ -2901,14 +2909,14 @@
         <v>41</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="7"/>
       <c r="E44" s="6"/>
       <c r="F44" s="6"/>
       <c r="G44" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H44" s="8"/>
       <c r="I44" s="9"/>
@@ -2920,7 +2928,7 @@
       <c r="L44" s="9"/>
       <c r="M44" s="9"/>
       <c r="N44" s="10" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="O44" s="9"/>
     </row>
@@ -2929,16 +2937,16 @@
         <v>42</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C45" s="6"/>
       <c r="D45" s="7"/>
       <c r="E45" s="6"/>
       <c r="F45" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H45" s="8"/>
       <c r="I45" s="9"/>
@@ -2950,7 +2958,7 @@
       <c r="L45" s="9"/>
       <c r="M45" s="9"/>
       <c r="N45" s="10" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O45" s="9"/>
     </row>
@@ -2959,20 +2967,20 @@
         <v>43</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D46" s="7"/>
       <c r="E46" s="6" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F46" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H46" s="8"/>
       <c r="I46" s="9"/>
@@ -2984,7 +2992,7 @@
       <c r="L46" s="9"/>
       <c r="M46" s="9"/>
       <c r="N46" s="10" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="O46" s="9"/>
     </row>
@@ -2993,16 +3001,16 @@
         <v>44</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
       <c r="E47" s="6"/>
       <c r="F47" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G47" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="H47" s="8"/>
       <c r="I47" s="9"/>
@@ -3014,7 +3022,7 @@
       <c r="L47" s="9"/>
       <c r="M47" s="9"/>
       <c r="N47" s="10" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="O47" s="9"/>
     </row>
@@ -3023,20 +3031,20 @@
         <v>45</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D48" s="7"/>
       <c r="E48" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F48" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="H48" s="8"/>
       <c r="I48" s="9"/>
@@ -3048,7 +3056,7 @@
       <c r="L48" s="9"/>
       <c r="M48" s="9"/>
       <c r="N48" s="10" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="O48" s="9"/>
     </row>
@@ -3057,20 +3065,20 @@
         <v>46</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D49" s="7"/>
       <c r="E49" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F49" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G49" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H49" s="8"/>
       <c r="I49" s="9"/>
@@ -3082,7 +3090,7 @@
       <c r="L49" s="9"/>
       <c r="M49" s="9"/>
       <c r="N49" s="10" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O49" s="9"/>
     </row>
@@ -3091,20 +3099,20 @@
         <v>47</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F50" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G50" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="H50" s="8"/>
       <c r="I50" s="9"/>
@@ -3116,7 +3124,7 @@
       <c r="L50" s="9"/>
       <c r="M50" s="9"/>
       <c r="N50" s="10" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="O50" s="9"/>
     </row>
@@ -3125,20 +3133,20 @@
         <v>48</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F51" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G51" s="6" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H51" s="8"/>
       <c r="I51" s="9"/>
@@ -3150,7 +3158,7 @@
       <c r="L51" s="9"/>
       <c r="M51" s="9"/>
       <c r="N51" s="10" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="O51" s="9"/>
     </row>
@@ -3159,16 +3167,16 @@
         <v>49</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C52" s="6"/>
       <c r="D52" s="7"/>
       <c r="E52" s="6"/>
       <c r="F52" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="H52" s="8"/>
       <c r="I52" s="9"/>
@@ -3180,7 +3188,7 @@
       <c r="L52" s="9"/>
       <c r="M52" s="9"/>
       <c r="N52" s="10" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="O52" s="9"/>
     </row>
@@ -3189,16 +3197,16 @@
         <v>50</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C53" s="6"/>
       <c r="D53" s="7"/>
       <c r="E53" s="6"/>
       <c r="F53" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G53" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="H53" s="8"/>
       <c r="I53" s="9"/>
@@ -3210,7 +3218,7 @@
       <c r="L53" s="9"/>
       <c r="M53" s="9"/>
       <c r="N53" s="10" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O53" s="9"/>
     </row>
@@ -3219,20 +3227,20 @@
         <v>51</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="6" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F54" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H54" s="8"/>
       <c r="I54" s="9"/>
@@ -3244,7 +3252,7 @@
       <c r="L54" s="9"/>
       <c r="M54" s="9"/>
       <c r="N54" s="10" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="O54" s="9"/>
     </row>
@@ -3253,20 +3261,20 @@
         <v>52</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D55" s="7"/>
       <c r="E55" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G55" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H55" s="8"/>
       <c r="I55" s="9"/>
@@ -3278,7 +3286,7 @@
       <c r="L55" s="9"/>
       <c r="M55" s="9"/>
       <c r="N55" s="10" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="O55" s="9"/>
     </row>
@@ -3287,18 +3295,18 @@
         <v>53</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D56" s="7"/>
       <c r="E56" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H56" s="8"/>
       <c r="I56" s="9"/>
@@ -3310,7 +3318,7 @@
       <c r="L56" s="9"/>
       <c r="M56" s="9"/>
       <c r="N56" s="10" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="O56" s="9"/>
     </row>
@@ -3319,18 +3327,18 @@
         <v>54</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D57" s="7"/>
       <c r="E57" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="H57" s="8"/>
       <c r="I57" s="9"/>
@@ -3342,7 +3350,7 @@
       <c r="L57" s="9"/>
       <c r="M57" s="9"/>
       <c r="N57" s="10" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="O57" s="9"/>
     </row>
@@ -3351,20 +3359,20 @@
         <v>55</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D58" s="7"/>
       <c r="E58" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="F58" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H58" s="8"/>
       <c r="I58" s="9"/>
@@ -3376,7 +3384,7 @@
       <c r="L58" s="9"/>
       <c r="M58" s="9"/>
       <c r="N58" s="10" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="O58" s="9"/>
     </row>
@@ -3385,20 +3393,20 @@
         <v>56</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="H59" s="8"/>
       <c r="I59" s="9"/>
@@ -3410,7 +3418,7 @@
       <c r="L59" s="9"/>
       <c r="M59" s="9"/>
       <c r="N59" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O59" s="9"/>
     </row>
@@ -3419,18 +3427,18 @@
         <v>57</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="D60" s="7"/>
       <c r="E60" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F60" s="6"/>
       <c r="G60" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="H60" s="8"/>
       <c r="I60" s="9"/>
@@ -3442,7 +3450,7 @@
       <c r="L60" s="9"/>
       <c r="M60" s="9"/>
       <c r="N60" s="10" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="O60" s="9"/>
     </row>
@@ -3451,20 +3459,20 @@
         <v>58</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="F61" s="6" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="H61" s="8"/>
       <c r="I61" s="9"/>
@@ -3476,7 +3484,7 @@
       <c r="L61" s="9"/>
       <c r="M61" s="9"/>
       <c r="N61" s="10" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="O61" s="9"/>
     </row>
@@ -3485,14 +3493,14 @@
         <v>59</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C62" s="6"/>
       <c r="D62" s="7"/>
       <c r="E62" s="6"/>
       <c r="F62" s="6"/>
       <c r="G62" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H62" s="8"/>
       <c r="I62" s="9"/>
@@ -3504,7 +3512,7 @@
       <c r="L62" s="9"/>
       <c r="M62" s="9"/>
       <c r="N62" s="10" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="O62" s="9"/>
     </row>
@@ -3513,14 +3521,14 @@
         <v>60</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="C63" s="6"/>
       <c r="D63" s="7"/>
       <c r="E63" s="6"/>
       <c r="F63" s="6"/>
       <c r="G63" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="H63" s="8"/>
       <c r="I63" s="9"/>
@@ -3532,7 +3540,7 @@
       <c r="L63" s="9"/>
       <c r="M63" s="9"/>
       <c r="N63" s="10" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="O63" s="9"/>
     </row>

</xml_diff>